<commit_message>
Upd v2.29 Finished 3fr shool2 part1
Закнчил 3 этаж стены шк 2 часть 1
</commit_message>
<xml_diff>
--- a/school_2/vor_spartac_2_walls.xlsx
+++ b/school_2/vor_spartac_2_walls.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="480" yWindow="30" windowWidth="19155" windowHeight="8520" tabRatio="822" firstSheet="5" activeTab="12"/>
+    <workbookView xWindow="480" yWindow="30" windowWidth="19155" windowHeight="8520" tabRatio="822" firstSheet="5" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="ВОР" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="спец 5с" sheetId="6" r:id="rId6"/>
     <sheet name="ВОР 4с" sheetId="8" r:id="rId7"/>
     <sheet name="спец 4с" sheetId="9" r:id="rId8"/>
-    <sheet name="ВОР 3э1ч" sheetId="10" r:id="rId9"/>
+    <sheet name="ВОР ч1э3" sheetId="10" r:id="rId9"/>
     <sheet name="Спец7с3э" sheetId="11" r:id="rId10"/>
     <sheet name="Спец6с3э" sheetId="12" r:id="rId11"/>
     <sheet name="Спец5с3э" sheetId="13" r:id="rId12"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="106">
   <si>
     <t>№ п.п.</t>
   </si>
@@ -337,6 +337,18 @@
   </si>
   <si>
     <t>3.035</t>
+  </si>
+  <si>
+    <t>Спецификация выполненных работ (7 секция)</t>
+  </si>
+  <si>
+    <t>Спецификация выполненных работ (6 секция)</t>
+  </si>
+  <si>
+    <t>Спецификация выполненных работ (5 секция)</t>
+  </si>
+  <si>
+    <t>Штукатурка стен  и базовая шпаклевка (4 секция)</t>
   </si>
 </sst>
 </file>
@@ -382,18 +394,12 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="28">
@@ -1038,7 +1044,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1711,7 +1717,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="86" t="s">
-        <v>21</v>
+        <v>102</v>
       </c>
       <c r="B1" s="86"/>
       <c r="C1" s="86"/>
@@ -1786,7 +1792,7 @@
       <c r="D6" s="10">
         <v>83.583314279999996</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="87">
         <f t="shared" ref="E6:E7" si="0">C6+D6</f>
         <v>95.483314280000002</v>
       </c>
@@ -1858,7 +1864,7 @@
       <c r="D10" s="10">
         <v>80.532918559999999</v>
       </c>
-      <c r="E10" s="10">
+      <c r="E10" s="87">
         <f t="shared" si="1"/>
         <v>138.99291855999999</v>
       </c>
@@ -1996,7 +2002,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="86" t="s">
-        <v>21</v>
+        <v>103</v>
       </c>
       <c r="B1" s="86"/>
       <c r="C1" s="86"/>
@@ -2245,7 +2251,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="86" t="s">
-        <v>21</v>
+        <v>104</v>
       </c>
       <c r="B1" s="86"/>
       <c r="C1" s="86"/>
@@ -2377,7 +2383,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="84" t="s">
-        <v>37</v>
+        <v>105</v>
       </c>
       <c r="B2" s="84"/>
       <c r="C2" s="84"/>

</xml_diff>